<commit_message>
Equipamentos: 1 fone JBL simples, MacBook Pro M1 Pro usado, HD 4 TB e SSD SanDisk 2 TB
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Me4XDFceywGg3W8EPqkQw6
</commit_message>
<xml_diff>
--- a/minerva/docs/minerva/equipamentos/Orcamento_Equipamentos_EJUP.xlsx
+++ b/minerva/docs/minerva/equipamentos/Orcamento_Equipamentos_EJUP.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1311,39 +1311,39 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Fone fechado Audio-Technica ATH-M20x</t>
+          <t>Fone JBL Tune 500 com fio</t>
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>560</v>
+        <v>135</v>
       </c>
       <c r="E22" s="8">
         <f>C22*D22</f>
-        <v>1120</v>
+        <v>135</v>
       </c>
       <c r="F22" s="7" t="n">
-        <v>487</v>
+        <v>116</v>
       </c>
       <c r="G22" s="8">
         <f>C22*F22</f>
-        <v>974</v>
+        <v>116</v>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>Mercado Livre, Pichau, Mundomax</t>
+          <t>Mercado Livre, Amazon, KaBuM</t>
         </is>
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>https://www.pichau.com.br/fone-de-ouvido-audio-technica-m20x-profissional-ath-m20x</t>
+          <t>https://www.zoom.com.br/fone-de-ouvido-e-headset/headphone-com-microfone-jbl-tune-500</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>Fechado: não vaza som para os microfones.</t>
+          <t>Com fio, para ouvir o gravador sem atraso. Versão sem fio (Tune 500BT) não serve para monitorar.</t>
         </is>
       </c>
     </row>
@@ -1875,125 +1875,279 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Edição</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>MacBook Pro 14" M1 Pro, 16 GB, 512 GB, usado em ótimo estado</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="7" t="n">
+        <v>7100</v>
+      </c>
+      <c r="E35" s="8">
+        <f>C35*D35</f>
+        <v>7100</v>
+      </c>
+      <c r="F35" s="7" t="n">
+        <v>5880</v>
+      </c>
+      <c r="G35" s="8">
+        <f>C35*F35</f>
+        <v>5880</v>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>Mac Switch e GGImports (seminovo com garantia); OLX e Mercado Livre (particular)</t>
+        </is>
+      </c>
+      <c r="I35" s="9" t="inlineStr">
+        <is>
+          <t>https://www.macswitch.com.br/products/macbook-pro-m1-pro-14</t>
+        </is>
+      </c>
+      <c r="J35" s="5" t="inlineStr">
+        <is>
+          <t>Seminovo com garantia de loja: R$ 6.900 a 7.500. Particular: R$ 5.000 a 9.500, sem garantia. Conferir saúde da bateria, ciclos, conta Apple desvinculada e carregador original.</t>
+        </is>
+      </c>
+    </row>
     <row r="36">
-      <c r="B36" s="10" t="inlineStr">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Edição</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>HD externo Seagate Expansion 4 TB (USB 3.0)</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>1190</v>
+      </c>
+      <c r="E36" s="8">
+        <f>C36*D36</f>
+        <v>1190</v>
+      </c>
+      <c r="F36" s="7" t="n">
+        <v>1115</v>
+      </c>
+      <c r="G36" s="8">
+        <f>C36*F36</f>
+        <v>1115</v>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>KaBuM, Amazon</t>
+        </is>
+      </c>
+      <c r="I36" s="9" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/1005358/hd-externo-portatil-seagate-expansion-4tb-2-5-usb-3-0-preto-stgx4000400</t>
+        </is>
+      </c>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>Para arquivo e backup. Para editar direto, o SSD é melhor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Edição</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>SSD externo SanDisk Portable 2 TB (800 MB/s, USB-C)</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>1900</v>
+      </c>
+      <c r="E37" s="8">
+        <f>C37*D37</f>
+        <v>1900</v>
+      </c>
+      <c r="F37" s="7" t="n">
+        <v>1859</v>
+      </c>
+      <c r="G37" s="8">
+        <f>C37*F37</f>
+        <v>1859</v>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>KaBuM</t>
+        </is>
+      </c>
+      <c r="I37" s="9" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/513298/ssd-externo-sandisk-2tb-800mbs-usb-portatil-grafite</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>No lugar do SanDisk de 560 MB/s: aquele é SSD interno SATA, precisa de case USB-C e sai mais caro (R$ 2.000 a 2.400). Este é externo, mais rápido e já liga no MacBook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="10" t="inlineStr">
         <is>
           <t>Total por categoria</t>
         </is>
       </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="11" t="n"/>
-      <c r="B37" s="12" t="inlineStr">
-        <is>
-          <t>Câmeras e lentes</t>
-        </is>
-      </c>
-      <c r="C37" s="11" t="n"/>
-      <c r="D37" s="11" t="n"/>
-      <c r="E37" s="13">
-        <f>SUMIF($A$6:$A$34,B37,$E$6:$E$34)</f>
-        <v>61145</v>
-      </c>
-      <c r="F37" s="11" t="n"/>
-      <c r="G37" s="13">
-        <f>SUMIF($A$6:$A$34,B37,$G$6:$G$34)</f>
-        <v>54032</v>
-      </c>
-      <c r="H37" s="11" t="n"/>
-      <c r="I37" s="11" t="n"/>
-      <c r="J37" s="11" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="11" t="n"/>
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>Áudio</t>
-        </is>
-      </c>
-      <c r="C38" s="11" t="n"/>
-      <c r="D38" s="11" t="n"/>
-      <c r="E38" s="13">
-        <f>SUMIF($A$6:$A$34,B38,$E$6:$E$34)</f>
-        <v>7144</v>
-      </c>
-      <c r="F38" s="11" t="n"/>
-      <c r="G38" s="13">
-        <f>SUMIF($A$6:$A$34,B38,$G$6:$G$34)</f>
-        <v>6100</v>
-      </c>
-      <c r="H38" s="11" t="n"/>
-      <c r="I38" s="11" t="n"/>
-      <c r="J38" s="11" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="11" t="n"/>
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>Iluminação</t>
-        </is>
-      </c>
-      <c r="C39" s="11" t="n"/>
-      <c r="D39" s="11" t="n"/>
-      <c r="E39" s="13">
-        <f>SUMIF($A$6:$A$34,B39,$E$6:$E$34)</f>
-        <v>6200</v>
-      </c>
-      <c r="F39" s="11" t="n"/>
-      <c r="G39" s="13">
-        <f>SUMIF($A$6:$A$34,B39,$G$6:$G$34)</f>
-        <v>5275</v>
-      </c>
-      <c r="H39" s="11" t="n"/>
-      <c r="I39" s="11" t="n"/>
-      <c r="J39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="11" t="n"/>
       <c r="B40" s="12" t="inlineStr">
         <is>
-          <t>Suporte e energia</t>
+          <t>Câmeras e lentes</t>
         </is>
       </c>
       <c r="C40" s="11" t="n"/>
       <c r="D40" s="11" t="n"/>
       <c r="E40" s="13">
-        <f>SUMIF($A$6:$A$34,B40,$E$6:$E$34)</f>
-        <v>2284</v>
+        <f>SUMIF($A$6:$A$37,B40,$E$6:$E$37)</f>
+        <v>61145</v>
       </c>
       <c r="F40" s="11" t="n"/>
       <c r="G40" s="13">
-        <f>SUMIF($A$6:$A$34,B40,$G$6:$G$34)</f>
-        <v>2122</v>
+        <f>SUMIF($A$6:$A$37,B40,$G$6:$G$37)</f>
+        <v>54032</v>
       </c>
       <c r="H40" s="11" t="n"/>
       <c r="I40" s="11" t="n"/>
       <c r="J40" s="11" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="14" t="n"/>
-      <c r="B41" s="15" t="inlineStr">
+      <c r="A41" s="11" t="n"/>
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>Áudio</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="n"/>
+      <c r="D41" s="11" t="n"/>
+      <c r="E41" s="13">
+        <f>SUMIF($A$6:$A$37,B41,$E$6:$E$37)</f>
+        <v>6159</v>
+      </c>
+      <c r="F41" s="11" t="n"/>
+      <c r="G41" s="13">
+        <f>SUMIF($A$6:$A$37,B41,$G$6:$G$37)</f>
+        <v>5242</v>
+      </c>
+      <c r="H41" s="11" t="n"/>
+      <c r="I41" s="11" t="n"/>
+      <c r="J41" s="11" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="n"/>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>Iluminação</t>
+        </is>
+      </c>
+      <c r="C42" s="11" t="n"/>
+      <c r="D42" s="11" t="n"/>
+      <c r="E42" s="13">
+        <f>SUMIF($A$6:$A$37,B42,$E$6:$E$37)</f>
+        <v>6200</v>
+      </c>
+      <c r="F42" s="11" t="n"/>
+      <c r="G42" s="13">
+        <f>SUMIF($A$6:$A$37,B42,$G$6:$G$37)</f>
+        <v>5275</v>
+      </c>
+      <c r="H42" s="11" t="n"/>
+      <c r="I42" s="11" t="n"/>
+      <c r="J42" s="11" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="11" t="n"/>
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>Suporte e energia</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="n"/>
+      <c r="D43" s="11" t="n"/>
+      <c r="E43" s="13">
+        <f>SUMIF($A$6:$A$37,B43,$E$6:$E$37)</f>
+        <v>2284</v>
+      </c>
+      <c r="F43" s="11" t="n"/>
+      <c r="G43" s="13">
+        <f>SUMIF($A$6:$A$37,B43,$G$6:$G$37)</f>
+        <v>2122</v>
+      </c>
+      <c r="H43" s="11" t="n"/>
+      <c r="I43" s="11" t="n"/>
+      <c r="J43" s="11" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="11" t="n"/>
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>Edição</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="n"/>
+      <c r="D44" s="11" t="n"/>
+      <c r="E44" s="13">
+        <f>SUMIF($A$6:$A$37,B44,$E$6:$E$37)</f>
+        <v>10190</v>
+      </c>
+      <c r="F44" s="11" t="n"/>
+      <c r="G44" s="13">
+        <f>SUMIF($A$6:$A$37,B44,$G$6:$G$37)</f>
+        <v>8854</v>
+      </c>
+      <c r="H44" s="11" t="n"/>
+      <c r="I44" s="11" t="n"/>
+      <c r="J44" s="11" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="n"/>
+      <c r="B45" s="15" t="inlineStr">
         <is>
           <t>TOTAL GERAL</t>
         </is>
       </c>
-      <c r="C41" s="14" t="n"/>
-      <c r="D41" s="14" t="n"/>
-      <c r="E41" s="16">
-        <f>SUM(E6:E34)</f>
-        <v>76773</v>
-      </c>
-      <c r="F41" s="14" t="n"/>
-      <c r="G41" s="16">
-        <f>SUM(G6:G34)</f>
-        <v>67529</v>
-      </c>
-      <c r="H41" s="14" t="n"/>
-      <c r="I41" s="14" t="n"/>
-      <c r="J41" s="14" t="n"/>
-    </row>
-    <row r="43">
-      <c r="B43" s="2" t="inlineStr">
+      <c r="C45" s="14" t="n"/>
+      <c r="D45" s="14" t="n"/>
+      <c r="E45" s="16">
+        <f>SUM(E6:E37)</f>
+        <v>85978</v>
+      </c>
+      <c r="F45" s="14" t="n"/>
+      <c r="G45" s="16">
+        <f>SUM(G6:G37)</f>
+        <v>75525</v>
+      </c>
+      <c r="H45" s="14" t="n"/>
+      <c r="I45" s="14" t="n"/>
+      <c r="J45" s="14" t="n"/>
+    </row>
+    <row r="47">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>Subtotal médio: média das lojas sérias pesquisadas. Subtotal menor: o menor preço visto, quase sempre no Pix ou em marketplace; serve de piso para negociação.</t>
         </is>
@@ -2030,6 +2184,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2041,7 +2198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2229,32 +2386,49 @@
     <row r="13">
       <c r="A13" s="18" t="inlineStr">
         <is>
-          <t>Importar dos EUA (B&amp;H, Adorama)</t>
+          <t>Mac Switch e GGImports</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Não compensa</t>
+          <t>MacBook seminovo</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Fora do Remessa Conforme: 60% de imposto mais ICMS. Uma FX30 de US$ 1.750 chegaria a cerca de R$ 18 mil, contra R$ 9,8 mil na Bella Photo.</t>
+          <t>Lojas de seminovos Apple com garantia (3 meses na Mac Switch) e troca em 7 dias. Particular na OLX sai mais barato, mas sem garantia: só comprar vendo a máquina ligada.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="18" t="inlineStr">
         <is>
+          <t>Importar dos EUA (B&amp;H, Adorama)</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Não compensa</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Fora do Remessa Conforme: 60% de imposto mais ICMS. Uma FX30 de US$ 1.750 chegaria a cerca de R$ 18 mil, contra R$ 9,8 mil na Bella Photo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
           <t>Trazer na mala</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Pode compensar em lente</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Cota de US$ 1.000; o excedente paga 50%. A Tamron 28-75 cabe na cota e economiza de R$ 1.000 a 1.500. Perde a garantia nacional.</t>
         </is>

</xml_diff>

<commit_message>
Equipamentos: microfones em suporte de mesa, sem braço articulado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Me4XDFceywGg3W8EPqkQw6
</commit_message>
<xml_diff>
--- a/minerva/docs/minerva/equipamentos/Orcamento_Equipamentos_EJUP.xlsx
+++ b/minerva/docs/minerva/equipamentos/Orcamento_Equipamentos_EJUP.xlsx
@@ -1223,39 +1223,39 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Braço articulado de mesa Fifine BM88</t>
+          <t>Suporte de mesa tipo tripé para microfone</t>
         </is>
       </c>
       <c r="C20" s="6" t="n">
         <v>4</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>300</v>
+        <v>55</v>
       </c>
       <c r="E20" s="8">
         <f>C20*D20</f>
-        <v>1200</v>
+        <v>220</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>260</v>
+        <v>47</v>
       </c>
       <c r="G20" s="8">
         <f>C20*F20</f>
-        <v>1040</v>
+        <v>188</v>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Pichau, Terabyte, KaBuM</t>
+          <t>Magalu, Amazon</t>
         </is>
       </c>
       <c r="I20" s="9" t="inlineStr">
         <is>
-          <t>https://www.pichau.com.br/braco-articulado-para-microfone-fifine-bm88-preto-bm88-blk</t>
+          <t>https://www.bondfaro.com.br/pedestal-para-microfone?page=2</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>Aguenta 1,5 kg, perfil baixo.</t>
+          <t>Como já é feito nos podcasts. O K688 costuma vir sem suporte: conferir no anúncio. Rosca 5/8" com adaptador para 3/8".</t>
         </is>
       </c>
     </row>
@@ -2047,12 +2047,12 @@
       <c r="D41" s="11" t="n"/>
       <c r="E41" s="13">
         <f>SUMIF($A$6:$A$37,B41,$E$6:$E$37)</f>
-        <v>6159</v>
+        <v>5179</v>
       </c>
       <c r="F41" s="11" t="n"/>
       <c r="G41" s="13">
         <f>SUMIF($A$6:$A$37,B41,$G$6:$G$37)</f>
-        <v>5242</v>
+        <v>4390</v>
       </c>
       <c r="H41" s="11" t="n"/>
       <c r="I41" s="11" t="n"/>
@@ -2135,12 +2135,12 @@
       <c r="D45" s="14" t="n"/>
       <c r="E45" s="16">
         <f>SUM(E6:E37)</f>
-        <v>85978</v>
+        <v>84998</v>
       </c>
       <c r="F45" s="14" t="n"/>
       <c r="G45" s="16">
         <f>SUM(G6:G37)</f>
-        <v>75525</v>
+        <v>74673</v>
       </c>
       <c r="H45" s="14" t="n"/>
       <c r="I45" s="14" t="n"/>

</xml_diff>